<commit_message>
Update ship cost model, loss parameters to 0, fix pipeline selection
</commit_message>
<xml_diff>
--- a/2026_project/2_data_processed/intermediate_output/combined_selected_manual_edit.xlsx
+++ b/2026_project/2_data_processed/intermediate_output/combined_selected_manual_edit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutka\MT\AdOpT-NET0_dw\2026_project\2_data_processed\intermediate_output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C22CB761-4EF8-4EF1-8ACC-FBF4D072F563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AA55CF-9FDD-4A1F-9AD6-38243B7C764A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1180" yWindow="0" windowWidth="23040" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10000" yWindow="2110" windowWidth="12220" windowHeight="7510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1041,6 +1041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:P145"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1098,7 +1099,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>15</v>
       </c>
@@ -1139,7 +1140,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>21</v>
       </c>
@@ -1180,7 +1181,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -1221,7 +1222,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>26</v>
       </c>
@@ -1262,7 +1263,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>28</v>
       </c>
@@ -1303,7 +1304,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>30</v>
       </c>
@@ -1344,7 +1345,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>32</v>
       </c>
@@ -1385,7 +1386,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>33</v>
       </c>
@@ -1426,7 +1427,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>35</v>
       </c>
@@ -1467,7 +1468,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>37</v>
       </c>
@@ -1508,7 +1509,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>39</v>
       </c>
@@ -1549,7 +1550,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>42</v>
       </c>
@@ -1590,7 +1591,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>43</v>
       </c>
@@ -1631,7 +1632,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>44</v>
       </c>
@@ -1672,7 +1673,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>45</v>
       </c>
@@ -1713,7 +1714,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>46</v>
       </c>
@@ -1754,7 +1755,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>47</v>
       </c>
@@ -1795,7 +1796,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>49</v>
       </c>
@@ -1836,7 +1837,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>50</v>
       </c>
@@ -1877,7 +1878,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>51</v>
       </c>
@@ -1918,7 +1919,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>52</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>53</v>
       </c>
@@ -2000,7 +2001,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>55</v>
       </c>
@@ -2041,7 +2042,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>56</v>
       </c>
@@ -2082,7 +2083,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -2123,7 +2124,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>58</v>
       </c>
@@ -2164,7 +2165,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>60</v>
       </c>
@@ -2205,7 +2206,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>61</v>
       </c>
@@ -2246,7 +2247,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>62</v>
       </c>
@@ -2287,7 +2288,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>63</v>
       </c>
@@ -2328,7 +2329,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>64</v>
       </c>
@@ -2369,7 +2370,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>65</v>
       </c>
@@ -2410,7 +2411,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>66</v>
       </c>
@@ -2451,7 +2452,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>68</v>
       </c>
@@ -2492,7 +2493,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>69</v>
       </c>
@@ -2533,7 +2534,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>70</v>
       </c>
@@ -2574,7 +2575,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
         <v>72</v>
       </c>
@@ -2615,7 +2616,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>73</v>
       </c>
@@ -2656,7 +2657,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" t="s">
         <v>74</v>
       </c>
@@ -2697,7 +2698,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>75</v>
       </c>
@@ -2738,7 +2739,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>76</v>
       </c>
@@ -2779,7 +2780,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>77</v>
       </c>
@@ -2820,7 +2821,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
         <v>78</v>
       </c>
@@ -2861,7 +2862,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
         <v>79</v>
       </c>
@@ -2902,7 +2903,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
         <v>81</v>
       </c>
@@ -2943,7 +2944,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>82</v>
       </c>
@@ -2984,7 +2985,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>84</v>
       </c>
@@ -3025,7 +3026,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
         <v>85</v>
       </c>
@@ -3066,7 +3067,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
         <v>86</v>
       </c>
@@ -3107,7 +3108,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>87</v>
       </c>
@@ -3148,7 +3149,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>88</v>
       </c>
@@ -3189,7 +3190,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>89</v>
       </c>
@@ -3230,7 +3231,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>91</v>
       </c>
@@ -3271,7 +3272,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
         <v>92</v>
       </c>
@@ -3312,7 +3313,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
         <v>93</v>
       </c>
@@ -3353,7 +3354,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>94</v>
       </c>
@@ -3394,7 +3395,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>95</v>
       </c>
@@ -3435,7 +3436,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
         <v>96</v>
       </c>
@@ -3476,7 +3477,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
         <v>97</v>
       </c>
@@ -3517,7 +3518,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
         <v>98</v>
       </c>
@@ -3558,7 +3559,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
         <v>99</v>
       </c>
@@ -3599,7 +3600,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
         <v>100</v>
       </c>
@@ -3640,7 +3641,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
         <v>101</v>
       </c>
@@ -3681,7 +3682,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="65" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
         <v>102</v>
       </c>
@@ -3722,7 +3723,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="66" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>103</v>
       </c>
@@ -3763,7 +3764,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>105</v>
       </c>
@@ -3804,7 +3805,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>106</v>
       </c>
@@ -3845,7 +3846,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>108</v>
       </c>
@@ -3886,7 +3887,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>109</v>
       </c>
@@ -3927,7 +3928,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
         <v>110</v>
       </c>
@@ -3968,7 +3969,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="72" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
         <v>111</v>
       </c>
@@ -4009,7 +4010,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" t="s">
         <v>112</v>
       </c>
@@ -4050,7 +4051,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="74" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" t="s">
         <v>114</v>
       </c>
@@ -4091,7 +4092,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" t="s">
         <v>115</v>
       </c>
@@ -4132,7 +4133,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B76" t="s">
         <v>116</v>
       </c>
@@ -4173,7 +4174,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
         <v>117</v>
       </c>
@@ -4214,7 +4215,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
         <v>118</v>
       </c>
@@ -4255,7 +4256,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
         <v>119</v>
       </c>
@@ -4296,7 +4297,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="80" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>120</v>
       </c>
@@ -4337,7 +4338,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B81" t="s">
         <v>122</v>
       </c>
@@ -4378,7 +4379,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B82" t="s">
         <v>123</v>
       </c>
@@ -4419,7 +4420,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B83" t="s">
         <v>124</v>
       </c>
@@ -4460,7 +4461,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B84" t="s">
         <v>125</v>
       </c>
@@ -4501,7 +4502,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B85" t="s">
         <v>127</v>
       </c>
@@ -4542,7 +4543,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B86" t="s">
         <v>129</v>
       </c>
@@ -4583,7 +4584,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B87" t="s">
         <v>130</v>
       </c>
@@ -4624,7 +4625,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B88" t="s">
         <v>131</v>
       </c>
@@ -4665,7 +4666,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B89" t="s">
         <v>132</v>
       </c>
@@ -4706,7 +4707,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>133</v>
       </c>
@@ -4741,7 +4742,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>137</v>
       </c>
@@ -4776,7 +4777,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>139</v>
       </c>
@@ -4811,7 +4812,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>142</v>
       </c>
@@ -4846,7 +4847,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>145</v>
       </c>
@@ -4881,7 +4882,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>148</v>
       </c>
@@ -4916,7 +4917,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>150</v>
       </c>
@@ -4951,7 +4952,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B97" t="s">
         <v>153</v>
       </c>
@@ -4980,7 +4981,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
         <v>156</v>
       </c>
@@ -5009,7 +5010,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B99" t="s">
         <v>157</v>
       </c>
@@ -5038,7 +5039,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B100" t="s">
         <v>158</v>
       </c>
@@ -5067,7 +5068,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B101" t="s">
         <v>159</v>
       </c>
@@ -5096,7 +5097,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B102" t="s">
         <v>160</v>
       </c>
@@ -5125,7 +5126,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B103" t="s">
         <v>161</v>
       </c>
@@ -5154,7 +5155,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B104" t="s">
         <v>163</v>
       </c>
@@ -5183,7 +5184,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B105" t="s">
         <v>164</v>
       </c>
@@ -5212,7 +5213,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B106" t="s">
         <v>166</v>
       </c>
@@ -5241,7 +5242,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B107" t="s">
         <v>167</v>
       </c>
@@ -5270,7 +5271,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B108" t="s">
         <v>74</v>
       </c>
@@ -5299,7 +5300,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B109" t="s">
         <v>168</v>
       </c>
@@ -5328,7 +5329,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B110" t="s">
         <v>169</v>
       </c>
@@ -5357,7 +5358,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="111" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B111" t="s">
         <v>79</v>
       </c>
@@ -5386,7 +5387,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="112" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B112" t="s">
         <v>93</v>
       </c>
@@ -5415,7 +5416,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B113" t="s">
         <v>170</v>
       </c>
@@ -5444,7 +5445,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B114" t="s">
         <v>171</v>
       </c>
@@ -5473,7 +5474,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="115" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B115" t="s">
         <v>172</v>
       </c>
@@ -5502,7 +5503,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="116" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B116" t="s">
         <v>173</v>
       </c>
@@ -5531,7 +5532,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="117" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B117" t="s">
         <v>174</v>
       </c>
@@ -5560,7 +5561,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="118" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B118" t="s">
         <v>175</v>
       </c>
@@ -5589,7 +5590,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="119" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B119" t="s">
         <v>176</v>
       </c>
@@ -5618,7 +5619,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="120" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B120" t="s">
         <v>177</v>
       </c>
@@ -5647,7 +5648,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="121" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B121" t="s">
         <v>178</v>
       </c>
@@ -5676,7 +5677,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="122" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B122" t="s">
         <v>179</v>
       </c>
@@ -5705,7 +5706,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="123" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B123" t="s">
         <v>180</v>
       </c>
@@ -5734,7 +5735,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="124" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B124" t="s">
         <v>181</v>
       </c>
@@ -5763,7 +5764,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="125" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B125" t="s">
         <v>182</v>
       </c>
@@ -5792,7 +5793,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="126" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B126" t="s">
         <v>183</v>
       </c>
@@ -5821,7 +5822,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B127" t="s">
         <v>184</v>
       </c>
@@ -5850,7 +5851,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B128" t="s">
         <v>185</v>
       </c>
@@ -5879,7 +5880,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="129" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B129" t="s">
         <v>186</v>
       </c>
@@ -5908,7 +5909,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="130" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B130" t="s">
         <v>187</v>
       </c>
@@ -5937,7 +5938,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="131" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B131" t="s">
         <v>188</v>
       </c>
@@ -5966,7 +5967,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="132" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B132" t="s">
         <v>189</v>
       </c>
@@ -5995,7 +5996,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="133" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B133" t="s">
         <v>190</v>
       </c>
@@ -6024,7 +6025,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="134" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B134" t="s">
         <v>191</v>
       </c>
@@ -6050,7 +6051,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="135" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B135" t="s">
         <v>192</v>
       </c>
@@ -6079,7 +6080,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="136" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B136" t="s">
         <v>193</v>
       </c>
@@ -6108,7 +6109,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="137" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B137" t="s">
         <v>117</v>
       </c>
@@ -6137,7 +6138,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="138" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B138" t="s">
         <v>194</v>
       </c>
@@ -6192,10 +6193,10 @@
         <v>20</v>
       </c>
       <c r="P139" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="140" spans="2:16" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="140" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B140" t="s">
         <v>127</v>
       </c>
@@ -6224,7 +6225,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="141" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B141" t="s">
         <v>196</v>
       </c>
@@ -6253,7 +6254,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="142" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B142" t="s">
         <v>99</v>
       </c>
@@ -6282,7 +6283,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="143" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
         <v>33</v>
       </c>
@@ -6311,7 +6312,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="144" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B144" t="s">
         <v>197</v>
       </c>
@@ -6340,7 +6341,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="145" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="B145" t="s">
         <v>198</v>
       </c>
@@ -6370,7 +6371,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P145" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P145" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Trieste"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="15">
+      <filters>
+        <filter val="Yes"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="P1:P1048576">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",P1)))</formula>

</xml_diff>